<commit_message>
data: cierre dia 2026-09-05_1535 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/Stock/stock_VSB_Cuyo.xlsx
+++ b/01_INPUTS/Stock/stock_VSB_Cuyo.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38FFF7FF-27CA-4C6C-AAFC-E5C377263DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C43A63DD-F1C9-41F3-A956-6F34C052AA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2904,7 +2904,7 @@
         <v>552</v>
       </c>
       <c r="J7">
-        <v>564</v>
+        <v>552</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -2916,7 +2916,7 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O7">
         <v>0</v>
@@ -2960,7 +2960,7 @@
         <v>90</v>
       </c>
       <c r="J8">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -2972,7 +2972,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O8">
         <v>0</v>
@@ -3016,7 +3016,7 @@
         <v>54</v>
       </c>
       <c r="J9">
-        <v>102</v>
+        <v>54</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3028,7 +3028,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="O9">
         <v>0</v>
@@ -3072,7 +3072,7 @@
         <v>396</v>
       </c>
       <c r="J10">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -3084,7 +3084,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O10">
         <v>0</v>
@@ -3576,7 +3576,7 @@
         <v>1080</v>
       </c>
       <c r="J19">
-        <v>1641</v>
+        <v>1620</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -3588,7 +3588,7 @@
         <v>0</v>
       </c>
       <c r="N19">
-        <v>561</v>
+        <v>540</v>
       </c>
       <c r="O19">
         <v>0</v>
@@ -3632,7 +3632,7 @@
         <v>1368</v>
       </c>
       <c r="J20">
-        <v>1371</v>
+        <v>1368</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -3644,7 +3644,7 @@
         <v>0</v>
       </c>
       <c r="N20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O20">
         <v>0</v>
@@ -4136,7 +4136,7 @@
         <v>597</v>
       </c>
       <c r="J29">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -4148,7 +4148,7 @@
         <v>0</v>
       </c>
       <c r="N29">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O29">
         <v>0</v>
@@ -4304,7 +4304,7 @@
         <v>210</v>
       </c>
       <c r="J32">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -4316,7 +4316,7 @@
         <v>0</v>
       </c>
       <c r="N32">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O32">
         <v>0</v>
@@ -4528,7 +4528,7 @@
         <v>502</v>
       </c>
       <c r="J36">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="K36">
         <v>0</v>
@@ -4540,7 +4540,7 @@
         <v>0</v>
       </c>
       <c r="N36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O36">
         <v>0</v>
@@ -4584,7 +4584,7 @@
         <v>1872</v>
       </c>
       <c r="J37">
-        <v>1884</v>
+        <v>1872</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -4596,7 +4596,7 @@
         <v>0</v>
       </c>
       <c r="N37">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O37">
         <v>0</v>
@@ -4637,22 +4637,22 @@
         <v>24</v>
       </c>
       <c r="I38">
+        <v>2328</v>
+      </c>
+      <c r="J38">
         <v>2334</v>
       </c>
-      <c r="J38">
-        <v>2358</v>
-      </c>
       <c r="K38">
         <v>0</v>
       </c>
       <c r="L38">
-        <v>2334</v>
+        <v>2328</v>
       </c>
       <c r="M38">
         <v>0</v>
       </c>
       <c r="N38">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="O38">
         <v>0</v>
@@ -4752,7 +4752,7 @@
         <v>84</v>
       </c>
       <c r="J40">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -4764,7 +4764,7 @@
         <v>0</v>
       </c>
       <c r="N40">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="O40">
         <v>0</v>
@@ -4805,22 +4805,22 @@
         <v>24</v>
       </c>
       <c r="I41">
+        <v>732</v>
+      </c>
+      <c r="J41">
         <v>738</v>
       </c>
-      <c r="J41">
-        <v>804</v>
-      </c>
       <c r="K41">
         <v>0</v>
       </c>
       <c r="L41">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="M41">
         <v>0</v>
       </c>
       <c r="N41">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="O41">
         <v>0</v>
@@ -4864,7 +4864,7 @@
         <v>183</v>
       </c>
       <c r="J42">
-        <v>207</v>
+        <v>183</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -4876,7 +4876,7 @@
         <v>0</v>
       </c>
       <c r="N42">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="O42">
         <v>0</v>
@@ -5480,7 +5480,7 @@
         <v>267</v>
       </c>
       <c r="J53">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -5492,7 +5492,7 @@
         <v>0</v>
       </c>
       <c r="N53">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O53">
         <v>0</v>
@@ -5648,7 +5648,7 @@
         <v>288</v>
       </c>
       <c r="J56">
-        <v>306</v>
+        <v>288</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -5660,7 +5660,7 @@
         <v>0</v>
       </c>
       <c r="N56">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="O56">
         <v>0</v>
@@ -5984,7 +5984,7 @@
         <v>27</v>
       </c>
       <c r="J62">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="K62">
         <v>0</v>
@@ -5996,7 +5996,7 @@
         <v>0</v>
       </c>
       <c r="N62">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O62">
         <v>0</v>
@@ -6040,7 +6040,7 @@
         <v>681</v>
       </c>
       <c r="J63">
-        <v>729</v>
+        <v>681</v>
       </c>
       <c r="K63">
         <v>0</v>
@@ -6052,7 +6052,7 @@
         <v>0</v>
       </c>
       <c r="N63">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="O63">
         <v>0</v>
@@ -6152,7 +6152,7 @@
         <v>416</v>
       </c>
       <c r="J65">
-        <v>533</v>
+        <v>416</v>
       </c>
       <c r="K65">
         <v>0</v>
@@ -6164,7 +6164,7 @@
         <v>0</v>
       </c>
       <c r="N65">
-        <v>117</v>
+        <v>0</v>
       </c>
       <c r="O65">
         <v>0</v>
@@ -6376,7 +6376,7 @@
         <v>497</v>
       </c>
       <c r="J69">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="K69">
         <v>0</v>
@@ -6388,7 +6388,7 @@
         <v>0</v>
       </c>
       <c r="N69">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O69">
         <v>0</v>
@@ -6432,7 +6432,7 @@
         <v>1785</v>
       </c>
       <c r="J70">
-        <v>1788</v>
+        <v>1785</v>
       </c>
       <c r="K70">
         <v>0</v>
@@ -6444,7 +6444,7 @@
         <v>0</v>
       </c>
       <c r="N70">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O70">
         <v>0</v>
@@ -6544,7 +6544,7 @@
         <v>141</v>
       </c>
       <c r="J72">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="K72">
         <v>0</v>
@@ -6556,7 +6556,7 @@
         <v>0</v>
       </c>
       <c r="N72">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O72">
         <v>0</v>
@@ -6656,7 +6656,7 @@
         <v>231</v>
       </c>
       <c r="J74">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="K74">
         <v>0</v>
@@ -6668,7 +6668,7 @@
         <v>0</v>
       </c>
       <c r="N74">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="O74">
         <v>0</v>
@@ -6712,7 +6712,7 @@
         <v>96</v>
       </c>
       <c r="J75">
-        <v>141</v>
+        <v>96</v>
       </c>
       <c r="K75">
         <v>0</v>
@@ -6724,7 +6724,7 @@
         <v>0</v>
       </c>
       <c r="N75">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="O75">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>958</v>
       </c>
       <c r="J77">
-        <v>970</v>
+        <v>958</v>
       </c>
       <c r="K77">
         <v>0</v>
@@ -6836,7 +6836,7 @@
         <v>0</v>
       </c>
       <c r="N77">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O77">
         <v>0</v>
@@ -7160,7 +7160,7 @@
         <v>62</v>
       </c>
       <c r="J83">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="K83">
         <v>0</v>
@@ -7172,7 +7172,7 @@
         <v>0</v>
       </c>
       <c r="N83">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O83">
         <v>0</v>
@@ -8112,7 +8112,7 @@
         <v>404</v>
       </c>
       <c r="J100">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="K100">
         <v>0</v>
@@ -8124,7 +8124,7 @@
         <v>0</v>
       </c>
       <c r="N100">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O100">
         <v>0</v>
@@ -9008,7 +9008,7 @@
         <v>168</v>
       </c>
       <c r="J116">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="K116">
         <v>0</v>
@@ -9020,7 +9020,7 @@
         <v>0</v>
       </c>
       <c r="N116">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O116">
         <v>0</v>
@@ -9064,7 +9064,7 @@
         <v>562</v>
       </c>
       <c r="J117">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="K117">
         <v>0</v>
@@ -9076,7 +9076,7 @@
         <v>0</v>
       </c>
       <c r="N117">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O117">
         <v>0</v>
@@ -9232,7 +9232,7 @@
         <v>198</v>
       </c>
       <c r="J120">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="K120">
         <v>0</v>
@@ -9244,7 +9244,7 @@
         <v>0</v>
       </c>
       <c r="N120">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O120">
         <v>0</v>
@@ -9786,7 +9786,7 @@
         <v>107</v>
       </c>
       <c r="J130">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="K130">
         <v>0</v>
@@ -9798,7 +9798,7 @@
         <v>0</v>
       </c>
       <c r="N130">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O130">
         <v>0</v>
@@ -10122,7 +10122,7 @@
         <v>138</v>
       </c>
       <c r="J136">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="K136">
         <v>0</v>
@@ -10134,7 +10134,7 @@
         <v>0</v>
       </c>
       <c r="N136">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O136">
         <v>0</v>
@@ -10738,7 +10738,7 @@
         <v>222</v>
       </c>
       <c r="J147">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="K147">
         <v>0</v>
@@ -10750,7 +10750,7 @@
         <v>0</v>
       </c>
       <c r="N147">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O147">
         <v>0</v>
@@ -10906,7 +10906,7 @@
         <v>186</v>
       </c>
       <c r="J150">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="K150">
         <v>0</v>
@@ -10918,7 +10918,7 @@
         <v>0</v>
       </c>
       <c r="N150">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O150">
         <v>0</v>
@@ -11242,7 +11242,7 @@
         <v>1968</v>
       </c>
       <c r="J156">
-        <v>1971</v>
+        <v>1968</v>
       </c>
       <c r="K156">
         <v>0</v>
@@ -11254,7 +11254,7 @@
         <v>0</v>
       </c>
       <c r="N156">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O156">
         <v>0</v>

</xml_diff>